<commit_message>
fix: harden lottery updates and accessibility
</commit_message>
<xml_diff>
--- a/台灣彩券分析報告.xlsx
+++ b/台灣彩券分析報告.xlsx
@@ -26,12 +26,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>更新時間</t>
+          <t>資料基準</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-28 01:00:14</t>
+          <t>大樂透 2026-07-24 第 115000073 期；威力彩 2026-07-27 第 115000060 期</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: update Taiwan Lottery draws
</commit_message>
<xml_diff>
--- a/台灣彩券分析報告.xlsx
+++ b/台灣彩券分析報告.xlsx
@@ -31,7 +31,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>大樂透 2026-07-24 第 115000073 期；威力彩 2026-07-27 第 115000060 期</t>
+          <t>大樂透 2026-07-28 第 115000074 期；威力彩 2026-07-27 第 115000060 期</t>
         </is>
       </c>
     </row>
@@ -47,7 +47,7 @@
         </is>
       </c>
       <c r="C3">
-        <v>115000073</v>
+        <v>115000074</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -56,7 +56,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -78,7 +78,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>12, 15, 16, 18, 29, 34</t>
+          <t>15, 16, 18, 19, 29, 34</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -251,7 +251,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>均衡分散</t>
+          <t>隨機基準</t>
         </is>
       </c>
       <c r="B4">
@@ -261,29 +261,29 @@
         <v>0.69</v>
       </c>
       <c r="D4">
-        <v>19.0</v>
+        <v>9.5</v>
       </c>
       <c r="E4">
-        <v>2.4</v>
+        <v>0.0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>近期趨勢</t>
+          <t>均衡分散</t>
         </is>
       </c>
       <c r="B5">
         <v>42</v>
       </c>
       <c r="C5">
-        <v>0.69</v>
+        <v>0.667</v>
       </c>
       <c r="D5">
-        <v>16.7</v>
+        <v>19.0</v>
       </c>
       <c r="E5">
         <v>2.4</v>
@@ -295,23 +295,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>隨機基準</t>
+          <t>近期趨勢</t>
         </is>
       </c>
       <c r="B6">
         <v>42</v>
       </c>
       <c r="C6">
-        <v>0.69</v>
+        <v>0.667</v>
       </c>
       <c r="D6">
-        <v>9.5</v>
+        <v>16.7</v>
       </c>
       <c r="E6">
-        <v>0.0</v>
+        <v>2.4</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -324,7 +324,7 @@
         <v>42</v>
       </c>
       <c r="C7">
-        <v>0.643</v>
+        <v>0.667</v>
       </c>
       <c r="D7">
         <v>11.9</v>
@@ -398,7 +398,7 @@
         <v>29</v>
       </c>
       <c r="C2">
-        <v>77.38</v>
+        <v>77.77</v>
       </c>
       <c r="D2">
         <v>10</v>
@@ -407,7 +407,7 @@
         <v>5</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G2">
         <v>100.0</v>
@@ -416,7 +416,7 @@
         <v>100.0</v>
       </c>
       <c r="I2">
-        <v>12.5</v>
+        <v>15.15</v>
       </c>
     </row>
     <row r="3">
@@ -424,28 +424,28 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C3">
-        <v>71.44</v>
+        <v>71.67</v>
       </c>
       <c r="D3">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E3">
         <v>4</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G3">
-        <v>100.0</v>
+        <v>80.0</v>
       </c>
       <c r="H3">
         <v>80.0</v>
       </c>
       <c r="I3">
-        <v>6.25</v>
+        <v>15.15</v>
       </c>
     </row>
     <row r="4">
@@ -453,28 +453,28 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C4">
-        <v>71.28</v>
+        <v>69.95</v>
       </c>
       <c r="D4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E4">
         <v>4</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>80.0</v>
+        <v>90.0</v>
       </c>
       <c r="H4">
         <v>80.0</v>
       </c>
       <c r="I4">
-        <v>12.5</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="5">
@@ -485,7 +485,7 @@
         <v>15</v>
       </c>
       <c r="C5">
-        <v>68.85</v>
+        <v>69.3</v>
       </c>
       <c r="D5">
         <v>7</v>
@@ -494,7 +494,7 @@
         <v>4</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
         <v>70.0</v>
@@ -503,7 +503,7 @@
         <v>80.0</v>
       </c>
       <c r="I5">
-        <v>0.0</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="6">
@@ -511,28 +511,28 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="C6">
-        <v>67.76</v>
+        <v>68.15</v>
       </c>
       <c r="D6">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G6">
-        <v>90.0</v>
+        <v>60.0</v>
       </c>
       <c r="H6">
-        <v>60.0</v>
+        <v>80.0</v>
       </c>
       <c r="I6">
-        <v>18.75</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="7">
@@ -540,28 +540,28 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="C7">
-        <v>67.7</v>
+        <v>68.13</v>
       </c>
       <c r="D7">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G7">
+        <v>90.0</v>
+      </c>
+      <c r="H7">
         <v>60.0</v>
       </c>
-      <c r="H7">
-        <v>80.0</v>
-      </c>
       <c r="I7">
-        <v>0.0</v>
+        <v>21.21</v>
       </c>
     </row>
     <row r="8">
@@ -572,7 +572,7 @@
         <v>11</v>
       </c>
       <c r="C8">
-        <v>67.21</v>
+        <v>67.58</v>
       </c>
       <c r="D8">
         <v>8</v>
@@ -581,7 +581,7 @@
         <v>3</v>
       </c>
       <c r="F8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G8">
         <v>80.0</v>
@@ -590,7 +590,7 @@
         <v>60.0</v>
       </c>
       <c r="I8">
-        <v>18.75</v>
+        <v>21.21</v>
       </c>
     </row>
     <row r="9">
@@ -601,7 +601,7 @@
         <v>4</v>
       </c>
       <c r="C9">
-        <v>66.82</v>
+        <v>67.22</v>
       </c>
       <c r="D9">
         <v>9</v>
@@ -610,7 +610,7 @@
         <v>3</v>
       </c>
       <c r="F9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G9">
         <v>90.0</v>
@@ -619,7 +619,7 @@
         <v>60.0</v>
       </c>
       <c r="I9">
-        <v>12.5</v>
+        <v>15.15</v>
       </c>
     </row>
     <row r="10">
@@ -627,28 +627,28 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="C10">
-        <v>66.74</v>
+        <v>67.03</v>
       </c>
       <c r="D10">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E10">
         <v>3</v>
       </c>
       <c r="F10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G10">
-        <v>80.0</v>
+        <v>70.0</v>
       </c>
       <c r="H10">
         <v>60.0</v>
       </c>
       <c r="I10">
-        <v>15.62</v>
+        <v>21.21</v>
       </c>
     </row>
     <row r="11">
@@ -656,28 +656,28 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="C11">
-        <v>66.66</v>
+        <v>66.86</v>
       </c>
       <c r="D11">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E11">
         <v>3</v>
       </c>
       <c r="F11">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G11">
-        <v>70.0</v>
+        <v>100.0</v>
       </c>
       <c r="H11">
         <v>60.0</v>
       </c>
       <c r="I11">
-        <v>18.75</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="12">
@@ -685,10 +685,10 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C12">
-        <v>66.36</v>
+        <v>64.95</v>
       </c>
       <c r="D12">
         <v>9</v>
@@ -697,7 +697,7 @@
         <v>3</v>
       </c>
       <c r="F12">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G12">
         <v>90.0</v>
@@ -706,7 +706,7 @@
         <v>60.0</v>
       </c>
       <c r="I12">
-        <v>9.38</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="13">
@@ -717,7 +717,7 @@
         <v>36</v>
       </c>
       <c r="C13">
-        <v>64.11</v>
+        <v>64.52</v>
       </c>
       <c r="D13">
         <v>6</v>
@@ -726,7 +726,7 @@
         <v>3</v>
       </c>
       <c r="F13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G13">
         <v>60.0</v>
@@ -735,7 +735,7 @@
         <v>60.0</v>
       </c>
       <c r="I13">
-        <v>9.38</v>
+        <v>12.12</v>
       </c>
     </row>
     <row r="14">
@@ -746,7 +746,7 @@
         <v>1</v>
       </c>
       <c r="C14">
-        <v>63.64</v>
+        <v>64.06</v>
       </c>
       <c r="D14">
         <v>6</v>
@@ -755,7 +755,7 @@
         <v>3</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14">
         <v>60.0</v>
@@ -764,7 +764,7 @@
         <v>60.0</v>
       </c>
       <c r="I14">
-        <v>6.25</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="15">
@@ -775,7 +775,7 @@
         <v>28</v>
       </c>
       <c r="C15">
-        <v>63.54</v>
+        <v>63.85</v>
       </c>
       <c r="D15">
         <v>7</v>
@@ -784,7 +784,7 @@
         <v>2</v>
       </c>
       <c r="F15">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G15">
         <v>70.0</v>
@@ -793,7 +793,7 @@
         <v>40.0</v>
       </c>
       <c r="I15">
-        <v>31.25</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="16">
@@ -804,7 +804,7 @@
         <v>35</v>
       </c>
       <c r="C16">
-        <v>62.7</v>
+        <v>63.15</v>
       </c>
       <c r="D16">
         <v>6</v>
@@ -813,7 +813,7 @@
         <v>3</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16">
         <v>60.0</v>
@@ -822,7 +822,7 @@
         <v>60.0</v>
       </c>
       <c r="I16">
-        <v>0.0</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="17">
@@ -830,28 +830,28 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="C17">
-        <v>62.21</v>
+        <v>62.7</v>
       </c>
       <c r="D17">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G17">
-        <v>80.0</v>
+        <v>60.0</v>
       </c>
       <c r="H17">
-        <v>40.0</v>
+        <v>60.0</v>
       </c>
       <c r="I17">
-        <v>18.75</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="18">
@@ -859,28 +859,28 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C18">
-        <v>60.81</v>
+        <v>62.03</v>
       </c>
       <c r="D18">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18">
         <v>2</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G18">
-        <v>80.0</v>
+        <v>70.0</v>
       </c>
       <c r="H18">
         <v>40.0</v>
       </c>
       <c r="I18">
-        <v>9.38</v>
+        <v>21.21</v>
       </c>
     </row>
     <row r="19">
@@ -888,28 +888,28 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C19">
-        <v>60.81</v>
+        <v>61.77</v>
       </c>
       <c r="D19">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E19">
         <v>2</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G19">
-        <v>80.0</v>
+        <v>90.0</v>
       </c>
       <c r="H19">
         <v>40.0</v>
       </c>
       <c r="I19">
-        <v>9.38</v>
+        <v>12.12</v>
       </c>
     </row>
     <row r="20">
@@ -917,13 +917,13 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C20">
-        <v>60.72</v>
+        <v>61.22</v>
       </c>
       <c r="D20">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E20">
         <v>2</v>
@@ -932,13 +932,13 @@
         <v>4</v>
       </c>
       <c r="G20">
-        <v>70.0</v>
+        <v>80.0</v>
       </c>
       <c r="H20">
         <v>40.0</v>
       </c>
       <c r="I20">
-        <v>12.5</v>
+        <v>12.12</v>
       </c>
     </row>
     <row r="21">
@@ -946,28 +946,28 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="C21">
-        <v>60.34</v>
+        <v>61.12</v>
       </c>
       <c r="D21">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E21">
         <v>2</v>
       </c>
       <c r="F21">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G21">
-        <v>80.0</v>
+        <v>70.0</v>
       </c>
       <c r="H21">
         <v>40.0</v>
       </c>
       <c r="I21">
-        <v>6.25</v>
+        <v>15.15</v>
       </c>
     </row>
     <row r="22">
@@ -975,28 +975,28 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="C22">
-        <v>59.94</v>
+        <v>60.67</v>
       </c>
       <c r="D22">
         <v>7</v>
       </c>
       <c r="E22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="G22">
         <v>70.0</v>
       </c>
       <c r="H22">
-        <v>20.0</v>
+        <v>40.0</v>
       </c>
       <c r="I22">
-        <v>40.62</v>
+        <v>12.12</v>
       </c>
     </row>
     <row r="23">
@@ -1004,28 +1004,28 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="C23">
-        <v>59.87</v>
+        <v>60.21</v>
       </c>
       <c r="D23">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E23">
         <v>2</v>
       </c>
       <c r="F23">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G23">
-        <v>80.0</v>
+        <v>70.0</v>
       </c>
       <c r="H23">
         <v>40.0</v>
       </c>
       <c r="I23">
-        <v>3.12</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="24">
@@ -1033,28 +1033,28 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="C24">
-        <v>59.79</v>
+        <v>60.21</v>
       </c>
       <c r="D24">
         <v>7</v>
       </c>
       <c r="E24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="G24">
         <v>70.0</v>
       </c>
       <c r="H24">
-        <v>40.0</v>
+        <v>20.0</v>
       </c>
       <c r="I24">
-        <v>6.25</v>
+        <v>42.42</v>
       </c>
     </row>
     <row r="25">
@@ -1065,25 +1065,25 @@
         <v>48</v>
       </c>
       <c r="C25">
-        <v>59.64</v>
+        <v>59.4</v>
       </c>
       <c r="D25">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E25">
         <v>1</v>
       </c>
       <c r="F25">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G25">
-        <v>90.0</v>
+        <v>80.0</v>
       </c>
       <c r="H25">
         <v>20.0</v>
       </c>
       <c r="I25">
-        <v>31.25</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="26">
@@ -1094,25 +1094,25 @@
         <v>47</v>
       </c>
       <c r="C26">
-        <v>58.31</v>
+        <v>58.13</v>
       </c>
       <c r="D26">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E26">
         <v>1</v>
       </c>
       <c r="F26">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G26">
-        <v>100.0</v>
+        <v>90.0</v>
       </c>
       <c r="H26">
         <v>20.0</v>
       </c>
       <c r="I26">
-        <v>18.75</v>
+        <v>21.21</v>
       </c>
     </row>
     <row r="27">
@@ -1123,7 +1123,7 @@
         <v>22</v>
       </c>
       <c r="C27">
-        <v>57.76</v>
+        <v>57.94</v>
       </c>
       <c r="D27">
         <v>7</v>
@@ -1132,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="F27">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G27">
         <v>70.0</v>
@@ -1141,7 +1141,7 @@
         <v>0.0</v>
       </c>
       <c r="I27">
-        <v>59.38</v>
+        <v>60.61</v>
       </c>
     </row>
     <row r="28">
@@ -1161,7 +1161,7 @@
         <v>0</v>
       </c>
       <c r="F28">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G28">
         <v>50.0</v>
@@ -1178,28 +1178,28 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C29">
-        <v>57.08</v>
+        <v>56.12</v>
       </c>
       <c r="D29">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E29">
         <v>0</v>
       </c>
       <c r="F29">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G29">
-        <v>60.0</v>
+        <v>70.0</v>
       </c>
       <c r="H29">
         <v>0.0</v>
       </c>
       <c r="I29">
-        <v>62.5</v>
+        <v>48.48</v>
       </c>
     </row>
     <row r="30">
@@ -1207,28 +1207,28 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="C30">
-        <v>55.88</v>
+        <v>55.21</v>
       </c>
       <c r="D30">
         <v>7</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="G30">
         <v>70.0</v>
       </c>
       <c r="H30">
-        <v>0.0</v>
+        <v>20.0</v>
       </c>
       <c r="I30">
-        <v>46.88</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="31">
@@ -1239,7 +1239,7 @@
         <v>13</v>
       </c>
       <c r="C31">
-        <v>54.59</v>
+        <v>54.98</v>
       </c>
       <c r="D31">
         <v>5</v>
@@ -1248,7 +1248,7 @@
         <v>2</v>
       </c>
       <c r="F31">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G31">
         <v>50.0</v>
@@ -1257,7 +1257,7 @@
         <v>40.0</v>
       </c>
       <c r="I31">
-        <v>15.62</v>
+        <v>18.18</v>
       </c>
     </row>
     <row r="32">
@@ -1265,7 +1265,7 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="C32">
         <v>53.85</v>
@@ -1297,7 +1297,7 @@
         <v>7</v>
       </c>
       <c r="C33">
-        <v>53.5</v>
+        <v>53.61</v>
       </c>
       <c r="D33">
         <v>5</v>
@@ -1306,7 +1306,7 @@
         <v>0</v>
       </c>
       <c r="F33">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G33">
         <v>50.0</v>
@@ -1315,7 +1315,7 @@
         <v>0.0</v>
       </c>
       <c r="I33">
-        <v>75.0</v>
+        <v>75.76</v>
       </c>
     </row>
     <row r="34">
@@ -1326,7 +1326,7 @@
         <v>20</v>
       </c>
       <c r="C34">
-        <v>52.88</v>
+        <v>53.16</v>
       </c>
       <c r="D34">
         <v>5</v>
@@ -1335,7 +1335,7 @@
         <v>1</v>
       </c>
       <c r="F34">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G34">
         <v>50.0</v>
@@ -1344,7 +1344,7 @@
         <v>20.0</v>
       </c>
       <c r="I34">
-        <v>37.5</v>
+        <v>39.39</v>
       </c>
     </row>
     <row r="35">
@@ -1352,28 +1352,28 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="C35">
-        <v>52.72</v>
+        <v>53.15</v>
       </c>
       <c r="D35">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F35">
         <v>1</v>
       </c>
       <c r="G35">
-        <v>50.0</v>
+        <v>60.0</v>
       </c>
       <c r="H35">
-        <v>40.0</v>
+        <v>20.0</v>
       </c>
       <c r="I35">
-        <v>3.12</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="36">
@@ -1384,7 +1384,7 @@
         <v>46</v>
       </c>
       <c r="C36">
-        <v>52.27</v>
+        <v>52.71</v>
       </c>
       <c r="D36">
         <v>4</v>
@@ -1393,7 +1393,7 @@
         <v>3</v>
       </c>
       <c r="F36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G36">
         <v>40.0</v>
@@ -1402,7 +1402,7 @@
         <v>60.0</v>
       </c>
       <c r="I36">
-        <v>3.12</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="37">
@@ -1413,7 +1413,7 @@
         <v>33</v>
       </c>
       <c r="C37">
-        <v>51.47</v>
+        <v>51.8</v>
       </c>
       <c r="D37">
         <v>5</v>
@@ -1422,7 +1422,7 @@
         <v>1</v>
       </c>
       <c r="F37">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G37">
         <v>50.0</v>
@@ -1431,7 +1431,7 @@
         <v>20.0</v>
       </c>
       <c r="I37">
-        <v>28.12</v>
+        <v>30.3</v>
       </c>
     </row>
     <row r="38">
@@ -1442,7 +1442,7 @@
         <v>17</v>
       </c>
       <c r="C38">
-        <v>48.19</v>
+        <v>48.61</v>
       </c>
       <c r="D38">
         <v>5</v>
@@ -1451,7 +1451,7 @@
         <v>1</v>
       </c>
       <c r="F38">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G38">
         <v>50.0</v>
@@ -1460,7 +1460,7 @@
         <v>20.0</v>
       </c>
       <c r="I38">
-        <v>6.25</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="39">
@@ -1471,7 +1471,7 @@
         <v>2</v>
       </c>
       <c r="C39">
-        <v>47.27</v>
+        <v>47.71</v>
       </c>
       <c r="D39">
         <v>4</v>
@@ -1480,7 +1480,7 @@
         <v>2</v>
       </c>
       <c r="F39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G39">
         <v>40.0</v>
@@ -1489,7 +1489,7 @@
         <v>40.0</v>
       </c>
       <c r="I39">
-        <v>3.12</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="40">
@@ -1497,7 +1497,7 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="C40">
         <v>46.8</v>
@@ -1529,7 +1529,7 @@
         <v>38</v>
       </c>
       <c r="C41">
-        <v>45.71</v>
+        <v>45.89</v>
       </c>
       <c r="D41">
         <v>4</v>
@@ -1538,7 +1538,7 @@
         <v>0</v>
       </c>
       <c r="F41">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G41">
         <v>40.0</v>
@@ -1547,7 +1547,7 @@
         <v>0.0</v>
       </c>
       <c r="I41">
-        <v>59.38</v>
+        <v>60.61</v>
       </c>
     </row>
     <row r="42">
@@ -1555,28 +1555,28 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C42">
-        <v>42.91</v>
+        <v>42.25</v>
       </c>
       <c r="D42">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E42">
         <v>1</v>
       </c>
       <c r="F42">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G42">
-        <v>30.0</v>
+        <v>40.0</v>
       </c>
       <c r="H42">
         <v>20.0</v>
       </c>
       <c r="I42">
-        <v>43.75</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="43">
@@ -1584,28 +1584,28 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="C43">
-        <v>42.91</v>
+        <v>41.8</v>
       </c>
       <c r="D43">
         <v>3</v>
       </c>
       <c r="E43">
+        <v>2</v>
+      </c>
+      <c r="F43">
         <v>1</v>
-      </c>
-      <c r="F43">
-        <v>14</v>
       </c>
       <c r="G43">
         <v>30.0</v>
       </c>
       <c r="H43">
-        <v>20.0</v>
+        <v>40.0</v>
       </c>
       <c r="I43">
-        <v>43.75</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="44">
@@ -1616,7 +1616,7 @@
         <v>9</v>
       </c>
       <c r="C44">
-        <v>41.51</v>
+        <v>41.8</v>
       </c>
       <c r="D44">
         <v>3</v>
@@ -1625,7 +1625,7 @@
         <v>1</v>
       </c>
       <c r="F44">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G44">
         <v>30.0</v>
@@ -1634,7 +1634,7 @@
         <v>20.0</v>
       </c>
       <c r="I44">
-        <v>34.38</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="45">
@@ -1642,25 +1642,25 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="C45">
-        <v>41.35</v>
+        <v>41.8</v>
       </c>
       <c r="D45">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E45">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45">
         <v>0</v>
       </c>
       <c r="G45">
-        <v>30.0</v>
+        <v>40.0</v>
       </c>
       <c r="H45">
-        <v>40.0</v>
+        <v>20.0</v>
       </c>
       <c r="I45">
         <v>0.0</v>
@@ -1671,10 +1671,10 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="C46">
-        <v>40.1</v>
+        <v>40.44</v>
       </c>
       <c r="D46">
         <v>3</v>
@@ -1683,7 +1683,7 @@
         <v>1</v>
       </c>
       <c r="F46">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G46">
         <v>30.0</v>
@@ -1692,7 +1692,7 @@
         <v>20.0</v>
       </c>
       <c r="I46">
-        <v>25.0</v>
+        <v>27.27</v>
       </c>
     </row>
     <row r="47">
@@ -1700,28 +1700,28 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="C47">
-        <v>40.1</v>
+        <v>39.99</v>
       </c>
       <c r="D47">
         <v>3</v>
       </c>
       <c r="E47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F47">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="G47">
         <v>30.0</v>
       </c>
       <c r="H47">
-        <v>20.0</v>
+        <v>0.0</v>
       </c>
       <c r="I47">
-        <v>25.0</v>
+        <v>57.58</v>
       </c>
     </row>
     <row r="48">
@@ -1729,28 +1729,28 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="C48">
-        <v>39.79</v>
+        <v>39.08</v>
       </c>
       <c r="D48">
         <v>3</v>
       </c>
       <c r="E48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F48">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="G48">
         <v>30.0</v>
       </c>
       <c r="H48">
-        <v>0.0</v>
+        <v>20.0</v>
       </c>
       <c r="I48">
-        <v>56.25</v>
+        <v>18.18</v>
       </c>
     </row>
     <row r="49">
@@ -1758,28 +1758,28 @@
         <v>48</v>
       </c>
       <c r="B49">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C49">
-        <v>38.69</v>
+        <v>38.17</v>
       </c>
       <c r="D49">
         <v>3</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F49">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G49">
         <v>30.0</v>
       </c>
       <c r="H49">
-        <v>20.0</v>
+        <v>0.0</v>
       </c>
       <c r="I49">
-        <v>15.62</v>
+        <v>45.45</v>
       </c>
     </row>
     <row r="50">
@@ -1790,7 +1790,7 @@
         <v>31</v>
       </c>
       <c r="C50">
-        <v>33.4</v>
+        <v>33.63</v>
       </c>
       <c r="D50">
         <v>2</v>
@@ -1799,7 +1799,7 @@
         <v>0</v>
       </c>
       <c r="F50">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G50">
         <v>20.0</v>
@@ -1808,7 +1808,7 @@
         <v>0.0</v>
       </c>
       <c r="I50">
-        <v>50.0</v>
+        <v>51.52</v>
       </c>
     </row>
   </sheetData>
@@ -1867,173 +1867,173 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>115000073</v>
+        <v>115000074</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D2">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E2">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F2">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G2">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H2">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I2">
-        <v>40</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>115000072</v>
+        <v>115000073</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E3">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F3">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="G3">
         <v>35</v>
       </c>
       <c r="H3">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I3">
-        <v>11</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>115000071</v>
+        <v>115000072</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E4">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F4">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G4">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="H4">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="I4">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>115000070</v>
+        <v>115000071</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="E5">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="F5">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="G5">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="H5">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="I5">
-        <v>7</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>115000069</v>
+        <v>115000070</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="C6">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="E6">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="F6">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="G6">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="H6">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I6">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>115000068</v>
+        <v>115000069</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="C7">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D7">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E7">
         <v>15</v>
@@ -2042,345 +2042,345 @@
         <v>18</v>
       </c>
       <c r="G7">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="H7">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="I7">
-        <v>37</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>115000067</v>
+        <v>115000068</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C8">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D8">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E8">
+        <v>15</v>
+      </c>
+      <c r="F8">
+        <v>18</v>
+      </c>
+      <c r="G8">
         <v>19</v>
       </c>
-      <c r="F8">
-        <v>23</v>
-      </c>
-      <c r="G8">
-        <v>39</v>
-      </c>
       <c r="H8">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="I8">
-        <v>15</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>115000066</v>
+        <v>115000067</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="C9">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D9">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E9">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F9">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="G9">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="H9">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I9">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>115000065</v>
+        <v>115000066</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="C10">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D10">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="E10">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F10">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="G10">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="H10">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>115000064</v>
+        <v>115000065</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="C11">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E11">
+        <v>23</v>
+      </c>
+      <c r="F11">
+        <v>24</v>
+      </c>
+      <c r="G11">
         <v>29</v>
       </c>
-      <c r="F11">
-        <v>33</v>
-      </c>
-      <c r="G11">
-        <v>34</v>
-      </c>
       <c r="H11">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I11">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>115000063</v>
+        <v>115000064</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="C12">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D12">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E12">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F12">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="G12">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H12">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="I12">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>115000062</v>
+        <v>115000063</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D13">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E13">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F13">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="G13">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="H13">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="I13">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>115000061</v>
+        <v>115000062</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E14">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F14">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="G14">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="H14">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="I14">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>115000060</v>
+        <v>115000061</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="C15">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="D15">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E15">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="F15">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="G15">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="H15">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="I15">
-        <v>31</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>115000059</v>
+        <v>115000060</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C16">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D16">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E16">
         <v>25</v>
       </c>
       <c r="F16">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="G16">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="H16">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I16">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>115000058</v>
+        <v>115000059</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="C17">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D17">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E17">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F17">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G17">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H17">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="I17">
-        <v>2</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18">
       <c r="A18">
-        <v>115000057</v>
+        <v>115000058</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="C18">
+        <v>8</v>
+      </c>
+      <c r="D18">
+        <v>9</v>
+      </c>
+      <c r="E18">
+        <v>16</v>
+      </c>
+      <c r="F18">
         <v>20</v>
-      </c>
-      <c r="D18">
-        <v>26</v>
-      </c>
-      <c r="E18">
-        <v>29</v>
-      </c>
-      <c r="F18">
-        <v>31</v>
       </c>
       <c r="G18">
         <v>37</v>
@@ -2389,810 +2389,810 @@
         <v>49</v>
       </c>
       <c r="I18">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19">
-        <v>115000056</v>
+        <v>115000057</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="C19">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="D19">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E19">
         <v>29</v>
       </c>
       <c r="F19">
+        <v>31</v>
+      </c>
+      <c r="G19">
         <v>37</v>
       </c>
-      <c r="G19">
-        <v>47</v>
-      </c>
       <c r="H19">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I19">
-        <v>11</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20">
       <c r="A20">
-        <v>115000055</v>
+        <v>115000056</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="C20">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D20">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E20">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F20">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="G20">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="H20">
         <v>48</v>
       </c>
       <c r="I20">
-        <v>30</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <v>115000054</v>
+        <v>115000055</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C21">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D21">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E21">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F21">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="G21">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="H21">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I21">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22">
       <c r="A22">
-        <v>115000053</v>
+        <v>115000054</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="C22">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D22">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="E22">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F22">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="G22">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="H22">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23">
       <c r="A23">
-        <v>115000052</v>
+        <v>115000053</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C23">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D23">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="E23">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F23">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="G23">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="H23">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="I23">
-        <v>34</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24">
-        <v>115000051</v>
+        <v>115000052</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C24">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D24">
+        <v>12</v>
+      </c>
+      <c r="E24">
         <v>18</v>
       </c>
-      <c r="E24">
-        <v>25</v>
-      </c>
       <c r="F24">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="G24">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="H24">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I24">
-        <v>48</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25">
       <c r="A25">
-        <v>115000050</v>
+        <v>115000051</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C25">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D25">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E25">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F25">
         <v>28</v>
       </c>
       <c r="G25">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="H25">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="I25">
-        <v>15</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26">
       <c r="A26">
-        <v>115000049</v>
+        <v>115000050</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="C26">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D26">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E26">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F26">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G26">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="H26">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="I26">
-        <v>45</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27">
       <c r="A27">
-        <v>115000048</v>
+        <v>115000049</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="C27">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D27">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E27">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F27">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G27">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="H27">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="I27">
-        <v>7</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28">
       <c r="A28">
-        <v>115000047</v>
+        <v>115000048</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="C28">
+        <v>6</v>
+      </c>
+      <c r="D28">
+        <v>10</v>
+      </c>
+      <c r="E28">
+        <v>14</v>
+      </c>
+      <c r="F28">
+        <v>25</v>
+      </c>
+      <c r="G28">
+        <v>26</v>
+      </c>
+      <c r="H28">
+        <v>32</v>
+      </c>
+      <c r="I28">
         <v>7</v>
-      </c>
-      <c r="D28">
-        <v>14</v>
-      </c>
-      <c r="E28">
-        <v>16</v>
-      </c>
-      <c r="F28">
-        <v>37</v>
-      </c>
-      <c r="G28">
-        <v>39</v>
-      </c>
-      <c r="H28">
-        <v>47</v>
-      </c>
-      <c r="I28">
-        <v>34</v>
       </c>
     </row>
     <row r="29">
       <c r="A29">
-        <v>115000046</v>
+        <v>115000047</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="C29">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D29">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E29">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F29">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="G29">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="H29">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="I29">
-        <v>22</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30">
       <c r="A30">
-        <v>115000045</v>
+        <v>115000046</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="C30">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D30">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E30">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F30">
+        <v>19</v>
+      </c>
+      <c r="G30">
+        <v>20</v>
+      </c>
+      <c r="H30">
+        <v>40</v>
+      </c>
+      <c r="I30">
         <v>22</v>
-      </c>
-      <c r="G30">
-        <v>40</v>
-      </c>
-      <c r="H30">
-        <v>45</v>
-      </c>
-      <c r="I30">
-        <v>18</v>
       </c>
     </row>
     <row r="31">
       <c r="A31">
-        <v>115000044</v>
+        <v>115000045</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="C31">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D31">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E31">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F31">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G31">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="H31">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="I31">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="32">
       <c r="A32">
-        <v>115000043</v>
+        <v>115000044</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="C32">
         <v>4</v>
       </c>
       <c r="D32">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E32">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F32">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="G32">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H32">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I32">
-        <v>30</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33">
       <c r="A33">
-        <v>115000042</v>
+        <v>115000043</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="C33">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D33">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E33">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F33">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G33">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H33">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="I33">
-        <v>47</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34">
       <c r="A34">
-        <v>115000041</v>
+        <v>115000042</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="C34">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D34">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E34">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F34">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="G34">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="H34">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="I34">
-        <v>8</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35">
       <c r="A35">
-        <v>115000040</v>
+        <v>115000041</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="C35">
         <v>5</v>
       </c>
       <c r="D35">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E35">
+        <v>13</v>
+      </c>
+      <c r="F35">
         <v>25</v>
       </c>
-      <c r="F35">
-        <v>40</v>
-      </c>
       <c r="G35">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="H35">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I35">
-        <v>39</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36">
       <c r="A36">
-        <v>115000039</v>
+        <v>115000040</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="C36">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D36">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E36">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F36">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="G36">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="H36">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="I36">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37">
       <c r="A37">
-        <v>115000038</v>
+        <v>115000039</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="C37">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="D37">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="E37">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="F37">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="G37">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="H37">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="I37">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="38">
       <c r="A38">
-        <v>115000037</v>
+        <v>115000038</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="C38">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D38">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="E38">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="F38">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G38">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H38">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="I38">
-        <v>21</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39">
       <c r="A39">
-        <v>115000036</v>
+        <v>115000037</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="C39">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D39">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E39">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="F39">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="G39">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H39">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I39">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40">
       <c r="A40">
-        <v>115000035</v>
+        <v>115000036</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="C40">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D40">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E40">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F40">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="G40">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="H40">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="I40">
-        <v>3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="41">
       <c r="A41">
-        <v>115000034</v>
+        <v>115000035</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="C41">
         <v>5</v>
       </c>
       <c r="D41">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E41">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F41">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G41">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H41">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I41">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42">
-        <v>115000033</v>
+        <v>115000034</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="C42">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D42">
         <v>11</v>
       </c>
       <c r="E42">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F42">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G42">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="H42">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="I42">
-        <v>42</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43">
       <c r="A43">
-        <v>115000032</v>
+        <v>115000033</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="C43">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D43">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E43">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F43">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="G43">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="H43">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="I43">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44">
       <c r="A44">
-        <v>115000031</v>
+        <v>115000032</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="C44">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="D44">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E44">
         <v>27</v>
       </c>
       <c r="F44">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="G44">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="H44">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="I44">
         <v>37</v>
@@ -3200,30 +3200,30 @@
     </row>
     <row r="45">
       <c r="A45">
-        <v>115000030</v>
+        <v>115000031</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="C45">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="D45">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="E45">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="F45">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="G45">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="H45">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="I45">
         <v>37</v>
@@ -3231,188 +3231,188 @@
     </row>
     <row r="46">
       <c r="A46">
-        <v>115000029</v>
+        <v>115000030</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="C46">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="D46">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="E46">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F46">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G46">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="H46">
         <v>49</v>
       </c>
       <c r="I46">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="47">
       <c r="A47">
-        <v>115000028</v>
+        <v>115000029</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="C47">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D47">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E47">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F47">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G47">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="H47">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I47">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="48">
       <c r="A48">
-        <v>115000027</v>
+        <v>115000028</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="C48">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="D48">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E48">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F48">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="G48">
+        <v>45</v>
+      </c>
+      <c r="H48">
         <v>47</v>
       </c>
-      <c r="H48">
+      <c r="I48">
         <v>48</v>
-      </c>
-      <c r="I48">
-        <v>7</v>
       </c>
     </row>
     <row r="49">
       <c r="A49">
-        <v>115000026</v>
+        <v>115000027</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="C49">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D49">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E49">
         <v>22</v>
       </c>
       <c r="F49">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="G49">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H49">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I49">
-        <v>31</v>
+        <v>7</v>
       </c>
     </row>
     <row r="50">
       <c r="A50">
-        <v>115000025</v>
+        <v>115000026</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="C50">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D50">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E50">
         <v>22</v>
       </c>
       <c r="F50">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="G50">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="H50">
+        <v>49</v>
+      </c>
+      <c r="I50">
         <v>31</v>
-      </c>
-      <c r="I50">
-        <v>45</v>
       </c>
     </row>
     <row r="51">
       <c r="A51">
-        <v>115000024</v>
+        <v>115000025</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="C51">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D51">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E51">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F51">
         <v>27</v>
       </c>
       <c r="G51">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="H51">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="I51">
-        <v>30</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>